<commit_message>
Works, now we have to simplify
</commit_message>
<xml_diff>
--- a/plants_data/CO2_Pipeline.xlsx
+++ b/plants_data/CO2_Pipeline.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\plants_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{355540A7-A3B5-48E2-8EE6-C14823D37B88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A7F6CDB-915D-475D-8EC8-8D0B493D52B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="distances" sheetId="2" r:id="rId1"/>

</xml_diff>